<commit_message>
feat: add maintenance demand calculation engine
</commit_message>
<xml_diff>
--- a/extensions/maintenance-api/templates/master_data_import_template.xlsx
+++ b/extensions/maintenance-api/templates/master_data_import_template.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="01_装备型号" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="02_构型版本" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="03_部件" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="04_维修器材" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="05_构型明细" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="06_可靠性参数" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="07_库房" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="08_库存" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="09_供应商" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="10_供应商报价" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_装备型号" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_构型版本" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_部件" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_维修器材" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_构型明细" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_可靠性参数" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_库房" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_库存" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_供应商" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_供应商报价" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_装备型号'!$A$1:$I$1</definedName>

</xml_diff>